<commit_message>
[feat] OrganizationData 추가 및 로드
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/FighterData.xlsx
+++ b/JsonConverter/ExcelFiles/FighterData.xlsx
@@ -19,44 +19,50 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+  <x:si>
+    <x:t>상대1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상대3</x:t>
+  </x:si>
   <x:si>
     <x:t>fighter_02</x:t>
   </x:si>
   <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 캐릭터이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Def</x:t>
+  </x:si>
+  <x:si>
     <x:t>Atk</x:t>
   </x:si>
   <x:si>
+    <x:t>김기본</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
     <x:t>Hp</x:t>
   </x:si>
   <x:si>
-    <x:t>김기본</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Def</x:t>
-  </x:si>
-  <x:si>
-    <x:t>김적</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 캐릭터이다</x:t>
+    <x:t>상대2</x:t>
   </x:si>
   <x:si>
     <x:t>float</x:t>
   </x:si>
   <x:si>
-    <x:t>기본 적이다</x:t>
-  </x:si>
-  <x:si>
     <x:t>(name)</x:t>
   </x:si>
   <x:si>
@@ -66,7 +72,19 @@
     <x:t>string</x:t>
   </x:si>
   <x:si>
-    <x:t>fighter_01</x:t>
+    <x:t>기본 상대2이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 상대1이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 상대3이다</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -852,58 +870,58 @@
   <x:sheetData>
     <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6" s="7" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C3" s="2" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F3" s="7" t="s">
         <x:v>7</x:v>
-      </x:c>
-      <x:c r="D3" s="7" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E3" s="7" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F3" s="7" t="s">
-        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>15</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>3</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>9</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D4" s="1">
         <x:v>100</x:v>
@@ -917,13 +935,13 @@
     </x:row>
     <x:row r="5" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="5" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="s">
-        <x:v>6</x:v>
-      </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>11</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D5" s="1">
         <x:v>150</x:v>
@@ -935,15 +953,45 @@
         <x:v>6</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A6" s="5"/>
-      <x:c r="B6" s="5"/>
-      <x:c r="C6" s="5"/>
-    </x:row>
-    <x:row r="7" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A7" s="5"/>
-      <x:c r="B7" s="5"/>
-      <x:c r="C7" s="5"/>
+    <x:row r="6" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A6" s="3" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D6" s="1">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="E6" s="1">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F6" s="1">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A7" s="3" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="5" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D7" s="1">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E7" s="1">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F7" s="1">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A8" s="5"/>

</xml_diff>

<commit_message>
[feat] MatchScheduleUI 닫기 구현 및 프리팹 정리
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/FighterData.xlsx
+++ b/JsonConverter/ExcelFiles/FighterData.xlsx
@@ -19,72 +19,99 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+  <x:si>
+    <x:t>fighter_05</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상대5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상대6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 캐릭터이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 상대2이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 상대1이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 상대3이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fighter_07</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상대2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상대3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hp</x:t>
+  </x:si>
   <x:si>
     <x:t>상대1</x:t>
   </x:si>
   <x:si>
-    <x:t>상대3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>fighter_02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 캐릭터이다</x:t>
-  </x:si>
-  <x:si>
-    <x:t>fighter_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
+    <x:t>김기본</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Atk</x:t>
   </x:si>
   <x:si>
     <x:t>Def</x:t>
   </x:si>
   <x:si>
-    <x:t>Atk</x:t>
-  </x:si>
-  <x:si>
-    <x:t>김기본</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>상대2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>float</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 상대2이다</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 상대1이다</x:t>
-  </x:si>
-  <x:si>
-    <x:t>fighter_03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>fighter_04</x:t>
-  </x:si>
-  <x:si>
-    <x:t>기본 상대3이다</x:t>
+    <x:t>상대4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 상대4이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 상대5이다</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 상대6이다</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -870,58 +897,58 @@
   <x:sheetData>
     <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6" s="7" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>10</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C3" s="2" t="s">
-        <x:v>3</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D3" s="7" t="s">
-        <x:v>11</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E3" s="7" t="s">
-        <x:v>8</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F3" s="7" t="s">
-        <x:v>7</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>9</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D4" s="1">
         <x:v>100</x:v>
@@ -935,13 +962,13 @@
     </x:row>
     <x:row r="5" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>0</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D5" s="1">
         <x:v>150</x:v>
@@ -955,13 +982,13 @@
     </x:row>
     <x:row r="6" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
-        <x:v>12</x:v>
-      </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D6" s="1">
         <x:v>170</x:v>
@@ -975,13 +1002,13 @@
     </x:row>
     <x:row r="7" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>21</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D7" s="1">
         <x:v>250</x:v>
@@ -993,17 +1020,66 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A8" s="5"/>
-      <x:c r="B8" s="5"/>
-      <x:c r="C8" s="5"/>
-    </x:row>
-    <x:row r="9" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A9" s="5"/>
-      <x:c r="B9" s="5"/>
-      <x:c r="C9" s="5"/>
-    </x:row>
-    <x:row r="10" ht="15.75" customHeight="1"/>
+    <x:row r="8" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A8" s="5" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D8" s="1">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="E8" s="1">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F8" s="1">
+        <x:v>15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A9" s="5" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="5" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D9" s="1">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="E9" s="1">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F9" s="1">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A10" s="1" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D10" s="1">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="E10" s="1">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F10" s="1">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
     <x:row r="11" ht="15.75" customHeight="1"/>
     <x:row r="12" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A12" s="6"/>

</xml_diff>